<commit_message>
correct data by adding monteverde and puerto jimenez cases/rr to calculations
</commit_message>
<xml_diff>
--- a/data/raw/dengue_limpio.xlsx
+++ b/data/raw/dengue_limpio.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://6f33fa7f78ea46e2aaca-my.sharepoint.com/personal/marianne_pena_ucr_ac_cr/Documents/cuenta personal/ucr pers/practica profesional/practica dengue/dengue-model/data/raw/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nan\OneDrive\Documentos\ucr\practica profesiona\dengue-model\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="224" documentId="8_{9CD5E471-BC98-4A0B-819A-C8C2CA15C75E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DA028A69-EC4B-48BD-98DF-D1DF0918CC56}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89697EEC-F5C4-4197-8ACE-780581371B5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="2" xr2:uid="{1E182B49-6C0E-4C8E-B74C-9692AEB1A419}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="5" xr2:uid="{1E182B49-6C0E-4C8E-B74C-9692AEB1A419}"/>
   </bookViews>
   <sheets>
     <sheet name="2020" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="581" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="180">
   <si>
     <t>TASA</t>
   </si>
@@ -61873,8 +61873,8 @@
       <c r="C74">
         <v>2709</v>
       </c>
-      <c r="D74">
-        <v>1859.1595692844055</v>
+      <c r="D74" t="s">
+        <v>42</v>
       </c>
       <c r="E74">
         <v>2</v>
@@ -77964,19 +77964,19 @@
         <v>163</v>
       </c>
       <c r="C74">
-        <v>722</v>
-      </c>
-      <c r="D74">
-        <v>489.47825143724918</v>
+        <v>727</v>
+      </c>
+      <c r="D74" t="s">
+        <v>42</v>
       </c>
       <c r="E74">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F74">
         <v>26</v>
       </c>
       <c r="G74">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H74">
         <v>36</v>
@@ -77985,7 +77985,7 @@
         <v>42</v>
       </c>
       <c r="J74">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K74">
         <v>24</v>
@@ -78060,7 +78060,7 @@
         <v>14</v>
       </c>
       <c r="AI74">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="AJ74">
         <v>9</v>
@@ -78087,7 +78087,7 @@
         <v>7</v>
       </c>
       <c r="AR74">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AS74">
         <v>11</v>
@@ -79002,10 +79002,10 @@
         <v>169</v>
       </c>
       <c r="C80">
-        <v>230</v>
-      </c>
-      <c r="D80">
-        <v>484.7922770482474</v>
+        <v>266</v>
+      </c>
+      <c r="D80" t="s">
+        <v>42</v>
       </c>
       <c r="E80">
         <v>0</v>
@@ -79014,10 +79014,10 @@
         <v>2</v>
       </c>
       <c r="G80">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H80">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I80">
         <v>0</v>
@@ -79032,10 +79032,10 @@
         <v>4</v>
       </c>
       <c r="M80">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N80">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O80">
         <v>1</v>
@@ -79083,73 +79083,73 @@
         <v>9</v>
       </c>
       <c r="AD80">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="AE80">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="AF80">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AG80">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AH80">
         <v>19</v>
       </c>
       <c r="AI80">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="AJ80">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AK80">
         <v>14</v>
       </c>
       <c r="AL80">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AM80">
         <v>7</v>
       </c>
       <c r="AN80">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="AO80">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AP80">
         <v>5</v>
       </c>
       <c r="AQ80">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AR80">
         <v>7</v>
       </c>
       <c r="AS80">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AT80">
         <v>6</v>
       </c>
       <c r="AU80">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="AV80">
         <v>9</v>
       </c>
       <c r="AW80">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AX80">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AY80">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AZ80">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="BA80">
         <v>4</v>
@@ -79161,7 +79161,7 @@
         <v>5</v>
       </c>
       <c r="BD80">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BE80">
         <v>0</v>
@@ -94057,10 +94057,10 @@
         <v>163</v>
       </c>
       <c r="C74">
-        <v>374</v>
-      </c>
-      <c r="D74">
-        <v>258.98662825724159</v>
+        <v>377</v>
+      </c>
+      <c r="D74" t="s">
+        <v>42</v>
       </c>
       <c r="E74">
         <v>1</v>
@@ -94165,7 +94165,7 @@
         <v>14</v>
       </c>
       <c r="AM74">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="AN74">
         <v>18</v>
@@ -94183,7 +94183,7 @@
         <v>12</v>
       </c>
       <c r="AS74">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="AT74">
         <v>11</v>
@@ -94213,7 +94213,7 @@
         <v>17</v>
       </c>
       <c r="BC74">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="BD74">
         <v>9</v>
@@ -95095,10 +95095,10 @@
         <v>169</v>
       </c>
       <c r="C80">
-        <v>34</v>
-      </c>
-      <c r="D80">
-        <v>106.28653599674888</v>
+        <v>42</v>
+      </c>
+      <c r="D80" t="s">
+        <v>42</v>
       </c>
       <c r="E80">
         <v>0</v>
@@ -95167,7 +95167,7 @@
         <v>0</v>
       </c>
       <c r="AA80">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB80">
         <v>0</v>
@@ -95188,10 +95188,10 @@
         <v>0</v>
       </c>
       <c r="AH80">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI80">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AJ80">
         <v>0</v>
@@ -95221,7 +95221,7 @@
         <v>1</v>
       </c>
       <c r="AS80">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AT80">
         <v>1</v>
@@ -95239,7 +95239,7 @@
         <v>2</v>
       </c>
       <c r="AY80">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AZ80">
         <v>1</v>
@@ -95254,7 +95254,7 @@
         <v>0</v>
       </c>
       <c r="BD80">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BE80">
         <v>0</v>

</xml_diff>